<commit_message>
BUS-629: roster + settings touch-ups from May 22 grading run
- Update BUS-629 Danh sách Nhóm.xlsx (minor roster edit)
- Append a few permission allowlist entries to .claude/settings.local.json
  picked up during Stage 1/2/4/5 grading and instructor PR pushes

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/courses/BUS-629-VEMBA-International-Corporate-Finance/BUS-629 Danh sách Nhóm.xlsx
+++ b/courses/BUS-629-VEMBA-International-Corporate-Finance/BUS-629 Danh sách Nhóm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\shidler\courses\BUS-629-VEMBA-International-Corporate-Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C534C6-6209-4983-B931-7BDD49512B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C5A18A-914C-4F8A-8316-3BDB0FADEFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'May 9-10 Breakouts'!$A$1:$C$24</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -244,15 +257,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -560,7 +573,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="2" max="2" width="27" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="40" customWidth="1"/>
   </cols>
   <sheetData>
@@ -571,7 +584,7 @@
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="7" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="8"/>
@@ -591,7 +604,7 @@
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="10" t="s">
         <v>5</v>
       </c>
       <c r="F3" s="8"/>
@@ -623,7 +636,7 @@
       <c r="B6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="10" t="s">
         <v>10</v>
       </c>
       <c r="F6" s="8"/>
@@ -655,7 +668,7 @@
       <c r="B9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="10" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="8"/>
@@ -687,7 +700,7 @@
       <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="10" t="s">
         <v>20</v>
       </c>
       <c r="F12" s="8"/>

</xml_diff>